<commit_message>
Fix API contract and add success report with UI improvements
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
   <si>
     <t xml:space="preserve">كود</t>
   </si>
@@ -65,6 +65,30 @@
   </si>
   <si>
     <t xml:space="preserve">BIO GAINERS CHOCOLATE 330 GM*10 SACHETS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73173</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONCOR 5 PLUS 30TAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOUX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOUX PROSPERITY SYRUP 120 ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73595</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIBRAX 30 TAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74881</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OCTOZINC CAP</t>
   </si>
 </sst>
 </file>
@@ -102,6 +126,7 @@
       <color theme="1"/>
       <name val="Noto Sans Devanagari"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -146,16 +171,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -351,101 +380,145 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10.14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="56.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="n">
+      <c r="C2" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="n">
+      <c r="A3" s="3" t="n">
         <v>74696</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="n">
+      <c r="A4" s="3" t="n">
         <v>73396</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="n">
+      <c r="A5" s="3" t="n">
         <v>17028</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="n">
+      <c r="A6" s="3" t="n">
         <v>10512</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="1" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update project files and add new report
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -1,21 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A655F402-3EF8-4A3D-BA0D-14783DB66301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="7"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,64 +20,94 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>كود</t>
-  </si>
-  <si>
-    <t>إسم الصنف</t>
-  </si>
-  <si>
-    <t>كمية النقص</t>
-  </si>
-  <si>
-    <t>إجمالي المبيعات</t>
-  </si>
-  <si>
-    <t>رصيد الادارة</t>
-  </si>
-  <si>
-    <t>رصيد العشرين</t>
-  </si>
-  <si>
-    <t>رصيد النجوم</t>
-  </si>
-  <si>
-    <t>رصيد الشهيد</t>
-  </si>
-  <si>
-    <t>رصيد العقبى</t>
-  </si>
-  <si>
-    <t>رصيد الوردانى</t>
-  </si>
-  <si>
-    <t>ACTI-COLLA ADVANCE 10 SACHET</t>
-  </si>
-  <si>
-    <t>ANTODINE 20 MG 3 AMP</t>
-  </si>
-  <si>
-    <t>AVIL 6 AMP</t>
-  </si>
-  <si>
-    <t>BETADINE SHAMPOO 120ML</t>
-  </si>
-  <si>
-    <t>BIO GAINERS CHOCOLATE 330 GM*10 SACHETS</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+  <si>
+    <t xml:space="preserve">كود</t>
+  </si>
+  <si>
+    <t xml:space="preserve">إسم الصنف</t>
+  </si>
+  <si>
+    <t xml:space="preserve">كمية النقص</t>
+  </si>
+  <si>
+    <t xml:space="preserve">إجمالي المبيعات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رصيد الادارة</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رصيد العشرين</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رصيد النجوم</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رصيد الشهيد</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رصيد العقبى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">رصيد الوردانى</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACTI-COLLA ADVANCE 10 SACHET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANTODINE 20 MG 3 AMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AVIL 6 AMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BETADINE SHAMPOO 120ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BIO GAINERS CHOCOLATE 330 GM*10 SACHETS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DANSET 8MG 3AMP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLOVERIN D 30 TAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEPOVIT B12 5 AMP</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="11"/>
@@ -101,7 +126,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -109,34 +134,58 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -178,12 +227,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -212,7 +261,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -233,7 +282,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -284,7 +333,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -302,33 +351,34 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J6"/>
-  <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultColWidth="8.57421875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="56.5703125" customWidth="1"/>
-    <col min="3" max="3" width="9.28515625" customWidth="1"/>
-    <col min="4" max="4" width="12.42578125" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" customWidth="1"/>
-    <col min="8" max="8" width="9.85546875" customWidth="1"/>
-    <col min="9" max="9" width="9.42578125" customWidth="1"/>
-    <col min="10" max="10" width="10.140625" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="9.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="10.14"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -360,60 +410,98 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+      <c r="C2" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2" t="n">
         <v>74696</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+      <c r="C3" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
         <v>73396</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+      <c r="C4" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
         <v>17028</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="C5" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
         <v>10512</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>75077</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>73366</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="0" t="n">
         <v>1</v>
       </c>
     </row>
   </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update configuration and core modules
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2343BF7A-6E66-463F-8054-E298B938B5B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F14CED-006B-4E05-8B14-014812705B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7200" yWindow="5850" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -395,7 +395,7 @@
         <v>10</v>
       </c>
       <c r="C2">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -406,7 +406,7 @@
         <v>11</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -417,7 +417,7 @@
         <v>12</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -428,7 +428,7 @@
         <v>13</v>
       </c>
       <c r="C5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -439,7 +439,7 @@
         <v>14</v>
       </c>
       <c r="C6">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -450,7 +450,7 @@
         <v>15</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -461,7 +461,7 @@
         <v>16</v>
       </c>
       <c r="C8">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -472,7 +472,7 @@
         <v>18</v>
       </c>
       <c r="C9">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Upload all local changes
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72F14CED-006B-4E05-8B14-014812705B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E08AF0-5238-4BD6-A30A-7D2967C21EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="5850" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>كود</t>
   </si>
@@ -100,6 +100,12 @@
   </si>
   <si>
     <t>NEUROTON 30 TABS</t>
+  </si>
+  <si>
+    <t>LIMITLESS MAN  MAX 100TAB</t>
+  </si>
+  <si>
+    <t>MELO OINT. 30 GM</t>
   </si>
 </sst>
 </file>
@@ -344,7 +350,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -483,7 +489,7 @@
         <v>19</v>
       </c>
       <c r="C10">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -494,7 +500,7 @@
         <v>21</v>
       </c>
       <c r="C11">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -505,7 +511,7 @@
         <v>22</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -516,7 +522,7 @@
         <v>23</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -525,6 +531,25 @@
       </c>
       <c r="B14" t="s">
         <v>24</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload remaining local changes
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E08AF0-5238-4BD6-A30A-7D2967C21EF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{483B2BDA-9BB2-4A4D-B9DD-CF565C82BC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -549,7 +549,7 @@
         <v>26</v>
       </c>
       <c r="C16">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refractoring file length end
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{483B2BDA-9BB2-4A4D-B9DD-CF565C82BC50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACFFFA2-EE7D-4EF8-A345-91E27334B078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1950" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t>كود</t>
   </si>
@@ -106,6 +106,12 @@
   </si>
   <si>
     <t>MELO OINT. 30 GM</t>
+  </si>
+  <si>
+    <t>36804</t>
+  </si>
+  <si>
+    <t>CEREBROLYSIN AMP 1ML</t>
   </si>
 </sst>
 </file>
@@ -350,7 +356,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr defaultColWidth="8.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -533,7 +539,7 @@
         <v>24</v>
       </c>
       <c r="C14">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -541,7 +547,7 @@
         <v>25</v>
       </c>
       <c r="C15">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -549,7 +555,18 @@
         <v>26</v>
       </c>
       <c r="C16">
-        <v>15</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
other fix for refractoring file length
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACFFFA2-EE7D-4EF8-A345-91E27334B078}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{460AFECF-8A49-4D3C-AB21-C5D13C4E4E87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -555,7 +555,7 @@
         <v>26</v>
       </c>
       <c r="C16">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -566,7 +566,7 @@
         <v>28</v>
       </c>
       <c r="C17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix same bug from  file organization plan
</commit_message>
<xml_diff>
--- a/data/input/order_items/shortage_report_total_20260622_error.xlsx
+++ b/data/input/order_items/shortage_report_total_20260622_error.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pyreview\PharmaSupplyBot\data\input\order_items\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F290D9A-12B1-4426-AF24-E2326C8522AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFD7278D-B35A-475E-AF5D-CC1B8493A56B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-16320" yWindow="-10410" windowWidth="16440" windowHeight="28320" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -650,7 +650,7 @@
         <v>30</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:9">
@@ -695,7 +695,7 @@
         <v>34</v>
       </c>
       <c r="C22">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:9">
@@ -706,7 +706,7 @@
         <v>36</v>
       </c>
       <c r="C23">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -717,7 +717,7 @@
         <v>38</v>
       </c>
       <c r="C24">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -739,7 +739,7 @@
         <v>42</v>
       </c>
       <c r="C26">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:9">
@@ -772,7 +772,7 @@
         <v>48</v>
       </c>
       <c r="C29">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>